<commit_message>
Central de avisos: fator R, limites de receita e recálculo quando a regra muda
O motor ganha avisos de fator R (com o ganho líquido de elevar o pró-labore)
e de proximidade dos limites do MEI, do Simples e do Presumido. A API reúne,
para a carteira toda, esses avisos, o possível imposto pago a mais em produtos
monofásicos e as simulações cujo resultado mudou com as regras atuais, e
recalcula cada uma criando uma nova versão (a anterior fica no histórico).
Tela de Avisos com filtros e a lista de mudanças na legislação, resumo no
painel, botão Recalcular no cliente e faixa com o antes e o depois.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVrp8HXiJ3fo8syeVkDidK
</commit_message>
<xml_diff>
--- a/validacao/casos_validacao.xlsx
+++ b/validacao/casos_validacao.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Alertas" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos'!$A$1:$I$284</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Casos'!$A$1:$I$291</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Memória de cálculo'!$A$1:$E$534</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 13/10/2026 com o motor tolaris_motor. 67 casos.</t>
+          <t>Gerado em 13/10/2026 com o motor tolaris_motor. 69 casos.</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I284"/>
+  <dimension ref="A1:I291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9845,10 +9845,234 @@
       <c r="H284" s="9" t="n"/>
       <c r="I284" s="10" t="n"/>
     </row>
+    <row r="285">
+      <c r="A285" s="13" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B285" s="13" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C285" s="14" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 60.000</t>
+        </is>
+      </c>
+      <c r="D285" s="13" t="inlineStr">
+        <is>
+          <t>DAS no Anexo V (fator R abaixo de 28%)</t>
+        </is>
+      </c>
+      <c r="E285" s="15" t="n">
+        <v>107100</v>
+      </c>
+      <c r="F285" s="8" t="n"/>
+      <c r="G285" s="15">
+        <f>IF(F285="","",E285-F285)</f>
+        <v/>
+      </c>
+      <c r="H285" s="13" t="n"/>
+      <c r="I285" s="14" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="13" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B286" s="13" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C286" s="14" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 60.000</t>
+        </is>
+      </c>
+      <c r="D286" s="13" t="inlineStr">
+        <is>
+          <t>DAS no Anexo III (fator R de 28%)</t>
+        </is>
+      </c>
+      <c r="E286" s="15" t="n">
+        <v>63360</v>
+      </c>
+      <c r="F286" s="8" t="n"/>
+      <c r="G286" s="15">
+        <f>IF(F286="","",E286-F286)</f>
+        <v/>
+      </c>
+      <c r="H286" s="13" t="n"/>
+      <c r="I286" s="14" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="13" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B287" s="13" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C287" s="14" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 60.000</t>
+        </is>
+      </c>
+      <c r="D287" s="13" t="inlineStr">
+        <is>
+          <t>INSS do sócio sobre o pró-labore adicional</t>
+        </is>
+      </c>
+      <c r="E287" s="15" t="n">
+        <v>475.2</v>
+      </c>
+      <c r="F287" s="8" t="n"/>
+      <c r="G287" s="15">
+        <f>IF(F287="","",E287-F287)</f>
+        <v/>
+      </c>
+      <c r="H287" s="13" t="n"/>
+      <c r="I287" s="14" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="13" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B288" s="13" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C288" s="14" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 60.000</t>
+        </is>
+      </c>
+      <c r="D288" s="13" t="inlineStr">
+        <is>
+          <t>Ganho líquido anual</t>
+        </is>
+      </c>
+      <c r="E288" s="15" t="n">
+        <v>43264.8</v>
+      </c>
+      <c r="F288" s="8" t="n"/>
+      <c r="G288" s="15">
+        <f>IF(F288="","",E288-F288)</f>
+        <v/>
+      </c>
+      <c r="H288" s="13" t="n"/>
+      <c r="I288" s="14" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="5" t="inlineStr">
+        <is>
+          <t>AV2</t>
+        </is>
+      </c>
+      <c r="B289" s="5" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C289" s="6" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 72.000</t>
+        </is>
+      </c>
+      <c r="D289" s="5" t="inlineStr">
+        <is>
+          <t>DAS no Anexo V (fator R abaixo de 28%)</t>
+        </is>
+      </c>
+      <c r="E289" s="7" t="n">
+        <v>107100</v>
+      </c>
+      <c r="F289" s="8" t="n"/>
+      <c r="G289" s="7">
+        <f>IF(F289="","",E289-F289)</f>
+        <v/>
+      </c>
+      <c r="H289" s="5" t="n"/>
+      <c r="I289" s="6" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="5" t="inlineStr">
+        <is>
+          <t>AV2</t>
+        </is>
+      </c>
+      <c r="B290" s="5" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C290" s="6" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 72.000</t>
+        </is>
+      </c>
+      <c r="D290" s="5" t="inlineStr">
+        <is>
+          <t>DAS no Anexo III (fator R de 28%)</t>
+        </is>
+      </c>
+      <c r="E290" s="7" t="n">
+        <v>63360</v>
+      </c>
+      <c r="F290" s="8" t="n"/>
+      <c r="G290" s="7">
+        <f>IF(F290="","",E290-F290)</f>
+        <v/>
+      </c>
+      <c r="H290" s="5" t="n"/>
+      <c r="I290" s="6" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="5" t="inlineStr">
+        <is>
+          <t>AV2</t>
+        </is>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>Avisos: fator R (2026)</t>
+        </is>
+      </c>
+      <c r="C291" s="6" t="inlineStr">
+        <is>
+          <t>Serviços com fator R; receita R$ 600.000; folha CLT R$ 96.000; pró-labore R$ 72.000</t>
+        </is>
+      </c>
+      <c r="D291" s="5" t="inlineStr">
+        <is>
+          <t>Impacto anual se cair para o Anexo V</t>
+        </is>
+      </c>
+      <c r="E291" s="7" t="n">
+        <v>43740</v>
+      </c>
+      <c r="F291" s="8" t="n"/>
+      <c r="G291" s="7">
+        <f>IF(F291="","",E291-F291)</f>
+        <v/>
+      </c>
+      <c r="H291" s="5" t="n"/>
+      <c r="I291" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I284"/>
+  <autoFilter ref="A1:I291"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185 H186 H187 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H202 H203 H204 H205 H206 H207 H208 H209 H210 H211 H212 H213 H214 H215 H216 H217 H218 H219 H220 H221 H222 H223 H224 H225 H226 H227 H228 H229 H230 H231 H232 H233 H234 H235 H236 H237 H238 H239 H240 H241 H242 H243 H244 H245 H246 H247 H248 H249 H250 H251 H252 H253 H254 H255 H256 H257 H258 H259 H260 H261 H262 H263 H264 H265 H266 H267 H268 H269 H270 H271 H272 H273 H274 H275 H276 H277 H278 H279 H280 H281 H282 H283 H284" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51 H52 H53 H54 H55 H56 H57 H58 H59 H60 H61 H62 H63 H64 H65 H66 H67 H68 H69 H70 H71 H72 H73 H74 H75 H76 H77 H78 H79 H80 H81 H82 H83 H84 H85 H86 H87 H88 H89 H90 H91 H92 H93 H94 H95 H96 H97 H98 H99 H100 H101 H102 H103 H104 H105 H106 H107 H108 H109 H110 H111 H112 H113 H114 H115 H116 H117 H118 H119 H120 H121 H122 H123 H124 H125 H126 H127 H128 H129 H130 H131 H132 H133 H134 H135 H136 H137 H138 H139 H140 H141 H142 H143 H144 H145 H146 H147 H148 H149 H150 H151 H152 H153 H154 H155 H156 H157 H158 H159 H160 H161 H162 H163 H164 H165 H166 H167 H168 H169 H170 H171 H172 H173 H174 H175 H176 H177 H178 H179 H180 H181 H182 H183 H184 H185 H186 H187 H188 H189 H190 H191 H192 H193 H194 H195 H196 H197 H198 H199 H200 H201 H202 H203 H204 H205 H206 H207 H208 H209 H210 H211 H212 H213 H214 H215 H216 H217 H218 H219 H220 H221 H222 H223 H224 H225 H226 H227 H228 H229 H230 H231 H232 H233 H234 H235 H236 H237 H238 H239 H240 H241 H242 H243 H244 H245 H246 H247 H248 H249 H250 H251 H252 H253 H254 H255 H256 H257 H258 H259 H260 H261 H262 H263 H264 H265 H266 H267 H268 H269 H270 H271 H272 H273 H274 H275 H276 H277 H278 H279 H280 H281 H282 H283 H284 H285 H286 H287 H288 H289 H290 H291" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Sim,Não,Revisar"</formula1>
     </dataValidation>
   </dataValidations>
@@ -23061,7 +23285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23740,6 +23964,30 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>Fator R de 27,28%: o cliente paga pelo Anexo V. Elevar o pró-labore em R$ 360,00 por mês leva o fator R a 28% e o DAS cai de R$ 107.100,00 para R$ 63.360,00 por ano. O INSS do sócio sobre o acréscimo custa cerca de R$ 475,20 por ano (supondo um sócio, antes do IRPF). Ganho líquido estimado: R$ 43.264,80 por ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>AV2</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Fator R de 29,28%, perto do mínimo de 28%. Sobram só R$ 7.680,00 de folha por ano acima do mínimo. Se a receita subir ou a folha cair, o cliente passa do Anexo III para o V e o DAS aumenta cerca de R$ 43.740,00 por ano (com a receita atual).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
README: enquadramento, CNAEs, tabelas do Simples de 2027 a 2033, legislação lida, kit de teste e fora do escopo; planilha de validação regenerada
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVrp8HXiJ3fo8syeVkDidK
</commit_message>
<xml_diff>
--- a/validacao/casos_validacao.xlsx
+++ b/validacao/casos_validacao.xlsx
@@ -553,7 +553,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Gerado em 13/10/2026 com o motor tolaris_motor. 69 casos.</t>
+          <t>Gerado em 26/10/2026 com o motor tolaris_motor. 69 casos.</t>
         </is>
       </c>
     </row>
@@ -18677,12 +18677,12 @@
       </c>
       <c r="B347" s="6" t="inlineStr">
         <is>
-          <t>Anexo I: alíquota efetiva do DAS</t>
+          <t>Anexo I: alíquota efetiva do DAS (2027)</t>
         </is>
       </c>
       <c r="C347" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 2.000.000,00</t>
+          <t>RBT12 R$ 2.000.000,00, 5ª faixa</t>
         </is>
       </c>
       <c r="D347" s="7" t="n">
@@ -18707,7 +18707,7 @@
       </c>
       <c r="C348" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,76% + COFINS 12,74% = 15,50% do DAS</t>
+          <t>CBS 15,33% + IBS 0,17% = 15,50% do DAS</t>
         </is>
       </c>
       <c r="D348" s="19" t="n">
@@ -18715,7 +18715,7 @@
       </c>
       <c r="E348" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -18827,12 +18827,12 @@
       </c>
       <c r="B353" s="6" t="inlineStr">
         <is>
-          <t>Anexo I: alíquota efetiva do DAS</t>
+          <t>Anexo I: alíquota efetiva do DAS (2033)</t>
         </is>
       </c>
       <c r="C353" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 2.000.000,00</t>
+          <t>RBT12 R$ 2.000.000,00, 5ª faixa</t>
         </is>
       </c>
       <c r="D353" s="7" t="n">
@@ -18857,7 +18857,7 @@
       </c>
       <c r="C354" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,76% + COFINS 12,74% + ICMS 33,50% = 49,00% do DAS</t>
+          <t>CBS 15,50% + IBS 33,50% = 49,00% do DAS</t>
         </is>
       </c>
       <c r="D354" s="19" t="n">
@@ -18865,7 +18865,7 @@
       </c>
       <c r="E354" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -18977,12 +18977,12 @@
       </c>
       <c r="B359" s="6" t="inlineStr">
         <is>
-          <t>Anexo III: alíquota efetiva do DAS</t>
+          <t>Anexo III: alíquota efetiva do DAS (2027)</t>
         </is>
       </c>
       <c r="C359" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 600.000,00</t>
+          <t>RBT12 R$ 600.000,00, 3ª faixa</t>
         </is>
       </c>
       <c r="D359" s="7" t="n">
@@ -19007,7 +19007,7 @@
       </c>
       <c r="C360" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,96% + COFINS 13,64% = 16,60% do DAS</t>
+          <t>CBS 16,41% + IBS 0,19% = 16,60% do DAS</t>
         </is>
       </c>
       <c r="D360" s="19" t="n">
@@ -19015,7 +19015,7 @@
       </c>
       <c r="E360" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -19127,12 +19127,12 @@
       </c>
       <c r="B365" s="6" t="inlineStr">
         <is>
-          <t>Anexo III: alíquota efetiva do DAS</t>
+          <t>Anexo III: alíquota efetiva do DAS (2033)</t>
         </is>
       </c>
       <c r="C365" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 600.000,00</t>
+          <t>RBT12 R$ 600.000,00, 3ª faixa</t>
         </is>
       </c>
       <c r="D365" s="7" t="n">
@@ -19157,7 +19157,7 @@
       </c>
       <c r="C366" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,96% + COFINS 13,64% + ISS 32,50% = 49,10% do DAS</t>
+          <t>CBS 16,60% + IBS 32,50% = 49,10% do DAS</t>
         </is>
       </c>
       <c r="D366" s="19" t="n">
@@ -19165,7 +19165,7 @@
       </c>
       <c r="E366" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -19277,12 +19277,12 @@
       </c>
       <c r="B371" s="6" t="inlineStr">
         <is>
-          <t>Anexo III: alíquota efetiva do DAS</t>
+          <t>Anexo III: alíquota efetiva do DAS (2027)</t>
         </is>
       </c>
       <c r="C371" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 1.200.000,00</t>
+          <t>RBT12 R$ 1.200.000,00, 4ª faixa</t>
         </is>
       </c>
       <c r="D371" s="7" t="n">
@@ -19307,7 +19307,7 @@
       </c>
       <c r="C372" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,96% + COFINS 13,64% = 16,60% do DAS</t>
+          <t>CBS 16,41% + IBS 0,19% = 16,60% do DAS</t>
         </is>
       </c>
       <c r="D372" s="19" t="n">
@@ -19315,7 +19315,7 @@
       </c>
       <c r="E372" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -19427,12 +19427,12 @@
       </c>
       <c r="B377" s="6" t="inlineStr">
         <is>
-          <t>Anexo III: alíquota efetiva do DAS</t>
+          <t>Anexo III: alíquota efetiva do DAS (2033)</t>
         </is>
       </c>
       <c r="C377" s="6" t="inlineStr">
         <is>
-          <t>RBT12 R$ 1.200.000,00</t>
+          <t>RBT12 R$ 1.200.000,00, 4ª faixa</t>
         </is>
       </c>
       <c r="D377" s="7" t="n">
@@ -19457,7 +19457,7 @@
       </c>
       <c r="C378" s="6" t="inlineStr">
         <is>
-          <t>PIS 2,96% + COFINS 13,64% + ISS 32,50% = 49,10% do DAS</t>
+          <t>CBS 16,60% + IBS 32,50% = 49,10% do DAS</t>
         </is>
       </c>
       <c r="D378" s="19" t="n">
@@ -19465,7 +19465,7 @@
       </c>
       <c r="E378" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, tabelas de partilha</t>
+          <t>Res. CGSN 190/2026, Anexos I a V (partilha)</t>
         </is>
       </c>
     </row>
@@ -23285,7 +23285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23312,7 +23312,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Fator R abaixo de 28%: acrescentar cerca de R$ 360,00/mês de pró-labore levaria ao Anexo III. Compare o custo do INSS sobre esse pró-labore.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
@@ -23324,50 +23324,50 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Fator R abaixo de 28%: acrescentar cerca de R$ 360,00/mês de pró-labore levaria ao Anexo III. Compare o custo do INSS sobre esse pró-labore.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>E1-LR</t>
+          <t>E1-SN</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>E2-SN</t>
+          <t>E1-LR</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>E2-LR</t>
+          <t>E2-SN</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>E3-SN</t>
+          <t>E2-SN</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -23379,79 +23379,79 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>E3-LR</t>
+          <t>E2-LR</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Prejuízo fiscal: IRPJ/CSLL zerados; o prejuízo compensa até 30% de lucros futuros.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>E3-LR</t>
+          <t>E3-SN</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>E4-SN</t>
+          <t>E3-LR</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Prejuízo fiscal: IRPJ/CSLL zerados; o prejuízo compensa até 30% de lucros futuros.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>E4-LR</t>
+          <t>E3-LR</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Prejuízo fiscal: IRPJ/CSLL zerados; o prejuízo compensa até 30% de lucros futuros.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>E4-LR</t>
+          <t>E4-SN</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>E5-SN</t>
+          <t>E4-LR</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Prejuízo fiscal: IRPJ/CSLL zerados; o prejuízo compensa até 30% de lucros futuros.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>E5-LR</t>
+          <t>E4-LR</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
@@ -23463,526 +23463,670 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>E6-SN</t>
+          <t>E5-SN</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Receita acima de R$ 4.800.000,00: empresa não pode optar pelo Simples.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>E6-LP</t>
+          <t>E5-LR</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Aplicado o acréscimo de 10% na presunção (LC 224/2025) sobre a receita acima de R$ 5 mi/ano. A regra é questionada no STF (ADIs 7920 e 7936) e há liminares afastando-a; confirme a situação do cliente.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>E6-LR</t>
+          <t>E6-SN</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Receita acima de R$ 4.800.000,00: empresa não pode optar pelo Simples Nacional.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>E7-SN</t>
+          <t>E6-LP</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Fator R abaixo de 28%: acrescentar cerca de R$ 10.500,00/mês de pró-labore levaria ao Anexo III. Compare o custo do INSS sobre esse pró-labore.</t>
+          <t>Aplicado o acréscimo de 10% na presunção (LC 224/2025) sobre a receita acima de R$ 5 mi/ano. A regra é questionada no STF (ADIs 7920 e 7936) e há liminares afastando-a; confirme a situação do cliente.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>E7-SN</t>
+          <t>E6-LR</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>E7-LR</t>
+          <t>E7-SN</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>SOC1-B</t>
+          <t>E7-SN</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
+          <t>Fator R abaixo de 28%: acrescentar cerca de R$ 10.500,00/mês de pró-labore levaria ao Anexo III. Compare o custo do INSS sobre esse pró-labore.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>SOC2-B</t>
+          <t>E7-SN</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>SOC3-B</t>
+          <t>E7-LR</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
+          <t>Estimativa gerencial: considera todo o estoque comprado como vendido no ano e não detalha adições/exclusões do LALUR além das informadas.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>SOC3-B</t>
+          <t>SOC1-B</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Renda anual acima de R$ 600 mil: sujeito ao IRPFM (alíquota mínima estimada de 6,00% sobre a renda total, abatido o IR já pago e o redutor de carga da PJ). Não incluído no custo mensal.</t>
+          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>RT1-2025</t>
+          <t>SOC2-B</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Premissas: vendas sem tributos mantidas em R$ 1.567.000,00/ano e aquisições com crédito em R$ 873.000,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
+          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>RT2-2025</t>
+          <t>SOC3-B</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Premissas: vendas sem tributos mantidas em R$ 1.096.200,00/ano e aquisições com crédito em R$ 108.900,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
+          <t>Dividendos pressupõem lucro contábil apurado (ou presumido menos tributos, sem escrituração) e distribuição aprovada.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>RT3-2025</t>
+          <t>SOC3-B</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Premissas: vendas sem tributos mantidas em R$ 548.100,00/ano e aquisições com crédito em R$ 54.450,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
+          <t>Renda anual acima de R$ 600 mil: sujeito ao IRPFM (alíquota mínima estimada de 6,00% sobre a renda total, abatido o IR já pago e o redutor de carga da PJ). Não incluído no custo mensal.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>RT4-2025</t>
+          <t>RT1-2025</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Premissas: vendas sem tributos mantidas em R$ 2.182.500,00/ano e aquisições com crédito em R$ 1.236.750,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
+          <t>Premissas: vendas sem tributos mantidas em R$ 1.567.000,00/ano e aquisições com crédito em R$ 873.000,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>SR1-2027</t>
+          <t>RT2-2025</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>Premissas: vendas sem tributos mantidas em R$ 1.096.200,00/ano e aquisições com crédito em R$ 108.900,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>SR1-2033</t>
+          <t>RT3-2025</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>2033: recolher por fora compensa mesmo sem vendas a empresas (créditos nas compras altos).</t>
+          <t>Premissas: vendas sem tributos mantidas em R$ 548.100,00/ano e aquisições com crédito em R$ 54.450,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>SR1-2033</t>
+          <t>RT4-2025</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>Premissas: vendas sem tributos mantidas em R$ 2.182.500,00/ano e aquisições com crédito em R$ 1.236.750,00/ano; alíquotas de referência CBS 8,8% e IBS 17,7% (estimativas — a de 2027 depende de TCU/Senado); Imposto Seletivo não incluído.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>SR2-2027</t>
+          <t>SR1-2027</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>SR2-2033</t>
+          <t>SR1-2027</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>SR3-2027</t>
+          <t>SR1-2033</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>2033: recolher por fora compensa mesmo sem vendas a empresas (créditos nas compras altos).</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>SR3-2033</t>
+          <t>SR1-2033</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>A partilha do DAS a partir de 2027 será redefinida (LC 214/2025); o cálculo usa a partilha atual como aproximação da fatia de IBS/CBS.</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>AU1-PF</t>
+          <t>SR1-2033</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>AU1-MEI</t>
+          <t>SR2-2027</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>O lucro do MEI acima da parcela isenta (receita x 32% em serviços, 8% em comércio, ou o lucro escriturado) entra na declaração anual de IRPF.</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>AU1-SN</t>
+          <t>SR2-2027</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>AU1-SN</t>
+          <t>SR2-2033</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 1.680,01.</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>AU2-PF</t>
+          <t>SR2-2033</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Livro-caixa só é dedutível para quem recebe de pessoas físicas e escritura as despesas; substitui o desconto simplificado quando for maior.</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>AU2-PF</t>
+          <t>SR3-2027</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>AU2-SN</t>
+          <t>SR3-2027</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>AU2-SN</t>
+          <t>SR3-2033</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 4.200,01.</t>
+          <t>O DAS e a fatia de IBS/CBS vêm dos Anexos da Res. CGSN 190/2026 para o ano (vigência a partir de 01/01/2027): CBS + IBS somam o que PIS, Cofins, ICMS e ISS somavam, exceto o IPI da indústria, que permanece; o teto de ISS cai de 5% (2027-28) a 3% (2032). O texto das tabelas foi lido nos autógrafos das leis e na Resolução; confirme na versão publicada.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>AU3-PF</t>
+          <t>SR3-2033</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
+          <t>Prazos de 2026 (Res. CGSN 186/2026, alterada pela 194/2026): a opção pelo regime regular de IBS/CBS para janeiro a junho de 2027 vai de 01/09 a 30/10/2026 e pode ser cancelada, em caráter irretratável, de 03/11 a 20/12/2026; as parcelas de IBS e CBS deixam de ser devidas no DAS. Empresas inscritas no CNPJ depois de 16/10 (Simples) ou de 31/10 (regime regular) seguem regra própria.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>AU3-SN</t>
+          <t>AU1-PF</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
+          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>AU3-SN</t>
+          <t>AU1-MEI</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 11.200,01.</t>
+          <t>O lucro do MEI acima da parcela isenta (receita x 32% em serviços, 8% em comércio, ou o lucro escriturado) entra na declaração anual de IRPF.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>REC1</t>
+          <t>AU1-SN</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>REC1</t>
+          <t>AU1-SN</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>REC1</t>
+          <t>AU1-SN</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 1.680,01.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>REC2</t>
+          <t>AU2-PF</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+          <t>Livro-caixa só é dedutível para quem recebe de pessoas físicas e escritura as despesas; substitui o desconto simplificado quando for maior.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>REC2</t>
+          <t>AU2-PF</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>REC2</t>
+          <t>AU2-SN</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>Em 2026-01 o ICMS já é recolhido fora do DAS (receita acima de R$ 3,6 milhões): não há economia de ICMS nesses meses.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>REC2</t>
+          <t>AU2-SN</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>REC3</t>
+          <t>AU2-SN</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 4.200,01.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>REC3</t>
+          <t>AU3-PF</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+          <t>Quem presta serviço a empresas tem 11% de INSS retido e a empresa paga mais 20% (custo para o cliente).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>REC3</t>
+          <t>AU3-SN</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+          <t>Folha do fator R (LC 123/2006, art. 18, §§ 24 a 26; Res. CGSN 140/2018, art. 26): remunerações pagas a pessoas físicas (com o 13º salário), pró-labore e FGTS; não entram aluguéis nem distribuição de lucros. A contribuição patronal só entra se for recolhida fora do DAS, o que não é o caso dos Anexos III e V. Se o valor apurado no eSocial ou no PGDAS-D for diferente, informe-o em "Folha do fator R informada".</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>AV1</t>
+          <t>AU3-SN</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Fator R de 27,28%: o cliente paga pelo Anexo V. Elevar o pró-labore em R$ 360,00 por mês leva o fator R a 28% e o DAS cai de R$ 107.100,00 para R$ 63.360,00 por ano. O INSS do sócio sobre o acréscimo custa cerca de R$ 475,20 por ano (supondo um sócio, antes do IRPF). Ganho líquido estimado: R$ 43.264,80 por ano.</t>
+          <t>Estimativa com faturamento mensal constante; o DAS real varia mês a mês com o RBT12.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
+          <t>AU3-SN</t>
+        </is>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Comparados pró-labore mínimo e pró-labore para fator R de 28%; escolhido: Anexo III, pró-labore de R$ 11.200,01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>REC1</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>REC1</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>REC1</t>
+        </is>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="inlineStr">
+        <is>
+          <t>REC2</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>REC2</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
+          <t>REC2</t>
+        </is>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Em 2026-01 o ICMS já é recolhido fora do DAS (receita acima de R$ 3,6 milhões): não há economia de ICMS nesses meses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>REC2</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="inlineStr">
+        <is>
+          <t>REC3</t>
+        </is>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Indício, não certeza: a estimativa supõe que a receita desses itens foi declarada no PGDAS-D sem segregação. Confira o que foi declarado em cada mês antes de retificar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>REC3</t>
+        </is>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>A lista de NCM é inicial e precisa ser conferida na tabela oficial da Receita Federal; o NCM completo (subitem) define se o produto é monofásico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>REC3</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Valores recolhidos a maior podem ser compensados ou restituídos em até 5 anos (CTN, art. 168); o cálculo cobre apenas o período importado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>AV1</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Fator R de 27,28%: o cliente paga pelo Anexo V. Elevar o pró-labore em R$ 360,00 por mês leva o fator R a 28% e o DAS cai de R$ 107.100,00 para R$ 63.360,00 por ano. O INSS do sócio sobre o acréscimo custa cerca de R$ 475,20 por ano (supondo um sócio, antes do IRPF). Ganho líquido estimado: R$ 43.264,80 por ano.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
           <t>AV2</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B70" s="6" t="inlineStr">
         <is>
           <t>Fator R de 29,28%, perto do mínimo de 28%. Sobram só R$ 7.680,00 de folha por ano acima do mínimo. Se a receita subir ou a folha cair, o cliente passa do Anexo III para o V e o DAS aumenta cerca de R$ 43.740,00 por ano (com a receita atual).</t>
         </is>

</xml_diff>

<commit_message>
Kit de teste leva a planilha de validação (85 casos); rótulo legível do INSS no Enquadramento
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVrp8HXiJ3fo8syeVkDidK
</commit_message>
<xml_diff>
--- a/validacao/casos_validacao.xlsx
+++ b/validacao/casos_validacao.xlsx
@@ -8008,7 +8008,7 @@
       </c>
       <c r="D227" s="5" t="inlineStr">
         <is>
-          <t>INSS do sócio sobre o pró-labore adicional (fator_r)</t>
+          <t>INSS do sócio sobre o pró-labore adicional (caminho do fator R)</t>
         </is>
       </c>
       <c r="E227" s="7" t="n">
@@ -8232,7 +8232,7 @@
       </c>
       <c r="D234" s="13" t="inlineStr">
         <is>
-          <t>INSS do sócio sobre o pró-labore adicional (fator_r)</t>
+          <t>INSS do sócio sobre o pró-labore adicional (caminho do fator R)</t>
         </is>
       </c>
       <c r="E234" s="15" t="n">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="D240" s="5" t="inlineStr">
         <is>
-          <t>INSS do sócio sobre o pró-labore adicional (fator_r)</t>
+          <t>INSS do sócio sobre o pró-labore adicional (caminho do fator R)</t>
         </is>
       </c>
       <c r="E240" s="7" t="n">
@@ -8808,7 +8808,7 @@
       </c>
       <c r="D252" s="13" t="inlineStr">
         <is>
-          <t>INSS do sócio sobre o pró-labore adicional (fator_r)</t>
+          <t>INSS do sócio sobre o pró-labore adicional (caminho do fator R)</t>
         </is>
       </c>
       <c r="E252" s="15" t="n">

</xml_diff>